<commit_message>
#6 R16 Updated in Schematic
</commit_message>
<xml_diff>
--- a/BOM/eSpark-BOM.xlsx
+++ b/BOM/eSpark-BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="354">
   <si>
     <t>Component list</t>
   </si>
@@ -360,9 +360,6 @@
     <t>RES SMD 4.7K OHM 5% 1/10W 0603</t>
   </si>
   <si>
-    <t>RES 5.6 OHM 1% 1/8W 0805</t>
-  </si>
-  <si>
     <t>RES 22 OHM 1% 1/10W 0603</t>
   </si>
   <si>
@@ -483,9 +480,6 @@
     <t>Res-0603</t>
   </si>
   <si>
-    <t>RES-0805</t>
-  </si>
-  <si>
     <t>Solder Bridge</t>
   </si>
   <si>
@@ -618,9 +612,6 @@
     <t>RC0603JR-074K7L</t>
   </si>
   <si>
-    <t>RC0805FR-075R6L</t>
-  </si>
-  <si>
     <t>RC0603FR-0722RL</t>
   </si>
   <si>
@@ -795,9 +786,6 @@
     <t>C277476</t>
   </si>
   <si>
-    <t>C441758</t>
-  </si>
-  <si>
     <t>C326057</t>
   </si>
   <si>
@@ -861,9 +849,6 @@
     <t>C105428</t>
   </si>
   <si>
-    <t>C275644</t>
-  </si>
-  <si>
     <t>C107701</t>
   </si>
   <si>
@@ -1074,7 +1059,28 @@
     <t>C1, C41, C43</t>
   </si>
   <si>
-    <t>R1, R6, R7, R8, R9, R10, R13, R14, R15, R31, R32</t>
+    <t>C0105C0G330J250NTZ</t>
+  </si>
+  <si>
+    <t>C881842</t>
+  </si>
+  <si>
+    <t>C15651</t>
+  </si>
+  <si>
+    <t>R1, R6, R7, R8, R10, R13, R14, R15, R31, R32</t>
+  </si>
+  <si>
+    <t>RES-1206</t>
+  </si>
+  <si>
+    <t>RC1206FR-7W5R6L</t>
+  </si>
+  <si>
+    <t>C137211</t>
+  </si>
+  <si>
+    <t>General Purpose Chip Resistor Thick Film 1206 5.6Ohm 1% Paper T/R</t>
   </si>
 </sst>
 </file>
@@ -1671,6 +1677,68 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1682,6 +1750,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1696,74 +1770,6 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2141,15 +2147,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="51"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="71"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2160,7 +2166,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="46" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2185,7 +2191,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="47" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -2199,7 +2205,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="52"/>
+      <c r="S3" s="72"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2210,7 +2216,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="47" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2224,7 +2230,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="53"/>
+      <c r="S4" s="73"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2249,7 +2255,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="53"/>
+      <c r="S5" s="73"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2270,7 +2276,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="53"/>
+      <c r="S6" s="73"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2291,7 +2297,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="53"/>
+      <c r="S7" s="73"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2312,7 +2318,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="53"/>
+      <c r="S8" s="73"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2329,46 +2335,46 @@
         <v>79</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H9" s="30" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>332</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>331</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>326</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>333</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>334</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>335</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="Q9" s="30" t="s">
         <v>337</v>
       </c>
-      <c r="J9" s="30" t="s">
-        <v>249</v>
-      </c>
-      <c r="K9" s="30" t="s">
-        <v>336</v>
-      </c>
-      <c r="L9" s="30" t="s">
-        <v>331</v>
-      </c>
-      <c r="M9" s="30" t="s">
+      <c r="R9" s="30" t="s">
         <v>338</v>
       </c>
-      <c r="N9" s="30" t="s">
+      <c r="S9" s="30" t="s">
         <v>339</v>
-      </c>
-      <c r="O9" s="30" t="s">
-        <v>340</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>341</v>
-      </c>
-      <c r="Q9" s="30" t="s">
-        <v>342</v>
-      </c>
-      <c r="R9" s="30" t="s">
-        <v>343</v>
-      </c>
-      <c r="S9" s="30" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2377,32 +2383,32 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="E10" s="37" t="s">
         <v>80</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="K10" s="37" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="L10" s="37">
         <v>3</v>
@@ -2414,8 +2420,8 @@
       <c r="N10" s="37">
         <v>50</v>
       </c>
-      <c r="O10" s="60" t="s">
-        <v>347</v>
+      <c r="O10" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P10" s="38">
         <v>1.89E-2</v>
@@ -2433,7 +2439,7 @@
         <f t="shared" ref="B11:B67" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="44" t="s">
@@ -2443,22 +2449,22 @@
         <v>81</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G11" s="44" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H11" s="44" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I11" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J11" s="44" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="K11" s="44" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="L11" s="44">
         <v>2</v>
@@ -2470,8 +2476,8 @@
       <c r="N11" s="44">
         <v>11</v>
       </c>
-      <c r="O11" s="61" t="s">
-        <v>347</v>
+      <c r="O11" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P11" s="45">
         <v>1.2122999999999999</v>
@@ -2489,7 +2495,7 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="37" t="s">
@@ -2499,22 +2505,22 @@
         <v>82</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="K12" s="37" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="L12" s="37">
         <v>14</v>
@@ -2526,8 +2532,8 @@
       <c r="N12" s="37">
         <v>100</v>
       </c>
-      <c r="O12" s="60" t="s">
-        <v>347</v>
+      <c r="O12" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P12" s="38">
         <v>5.0000000000000001E-3</v>
@@ -2545,7 +2551,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="44" t="s">
@@ -2555,22 +2561,22 @@
         <v>83</v>
       </c>
       <c r="F13" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G13" s="44" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H13" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I13" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J13" s="44" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="K13" s="44" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="L13" s="44">
         <v>1</v>
@@ -2582,8 +2588,8 @@
       <c r="N13" s="44">
         <v>100</v>
       </c>
-      <c r="O13" s="61" t="s">
-        <v>347</v>
+      <c r="O13" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P13" s="45">
         <v>2.8E-3</v>
@@ -2601,7 +2607,7 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="37" t="s">
@@ -2611,22 +2617,22 @@
         <v>84</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="K14" s="37" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="L14" s="37">
         <v>25</v>
@@ -2638,8 +2644,8 @@
       <c r="N14" s="37">
         <v>200</v>
       </c>
-      <c r="O14" s="60" t="s">
-        <v>347</v>
+      <c r="O14" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P14" s="38">
         <v>1.8E-3</v>
@@ -2657,7 +2663,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="44" t="s">
@@ -2667,22 +2673,22 @@
         <v>85</v>
       </c>
       <c r="F15" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G15" s="44" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H15" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I15" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J15" s="44" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="K15" s="44" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="L15" s="44">
         <v>2</v>
@@ -2694,8 +2700,8 @@
       <c r="N15" s="44">
         <v>15</v>
       </c>
-      <c r="O15" s="61" t="s">
-        <v>347</v>
+      <c r="O15" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P15" s="45">
         <v>0.16370000000000001</v>
@@ -2713,7 +2719,7 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="37" t="s">
@@ -2723,22 +2729,22 @@
         <v>86</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="L16" s="37">
         <v>2</v>
@@ -2750,8 +2756,8 @@
       <c r="N16" s="37">
         <v>15</v>
       </c>
-      <c r="O16" s="60" t="s">
-        <v>347</v>
+      <c r="O16" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P16" s="38">
         <v>0.42320000000000002</v>
@@ -2769,7 +2775,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="44" t="s">
@@ -2779,22 +2785,22 @@
         <v>87</v>
       </c>
       <c r="F17" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G17" s="44" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H17" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J17" s="44" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="K17" s="44" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="L17" s="44">
         <v>6</v>
@@ -2806,8 +2812,8 @@
       <c r="N17" s="44">
         <v>40</v>
       </c>
-      <c r="O17" s="61" t="s">
-        <v>347</v>
+      <c r="O17" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P17" s="45">
         <v>2.3800000000000002E-2</v>
@@ -2825,7 +2831,7 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="58" t="s">
+      <c r="C18" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="37" t="s">
@@ -2835,20 +2841,22 @@
         <v>88</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>141</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>178</v>
+        <v>140</v>
+      </c>
+      <c r="G18" s="54" t="s">
+        <v>176</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>225</v>
-      </c>
-      <c r="I18" s="37"/>
+        <v>222</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>346</v>
+      </c>
       <c r="J18" s="37" t="s">
-        <v>258</v>
+        <v>347</v>
       </c>
       <c r="K18" s="37" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="L18" s="37">
         <v>3</v>
@@ -2857,12 +2865,18 @@
         <f>L18*5</f>
         <v>15</v>
       </c>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="38"/>
+      <c r="N18" s="37">
+        <v>50</v>
+      </c>
+      <c r="O18" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="P18" s="38">
+        <v>5.4999999999999997E-3</v>
+      </c>
       <c r="Q18" s="38">
         <f>P18*N18</f>
-        <v>0</v>
+        <v>0.27499999999999997</v>
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="49"/>
@@ -2873,7 +2887,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D19" s="44" t="s">
@@ -2883,22 +2897,22 @@
         <v>89</v>
       </c>
       <c r="F19" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G19" s="44" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H19" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I19" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J19" s="44" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="K19" s="44" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="L19" s="44">
         <v>1</v>
@@ -2910,8 +2924,8 @@
       <c r="N19" s="44">
         <v>20</v>
       </c>
-      <c r="O19" s="61" t="s">
-        <v>347</v>
+      <c r="O19" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P19" s="45">
         <v>2.0199999999999999E-2</v>
@@ -2929,7 +2943,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D20" s="44" t="s">
@@ -2939,22 +2953,22 @@
         <v>90</v>
       </c>
       <c r="F20" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G20" s="44" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H20" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I20" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J20" s="44" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="K20" s="44" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="L20" s="44">
         <v>2</v>
@@ -2966,8 +2980,8 @@
       <c r="N20" s="44">
         <v>100</v>
       </c>
-      <c r="O20" s="61" t="s">
-        <v>347</v>
+      <c r="O20" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P20" s="45">
         <v>3.7000000000000002E-3</v>
@@ -2985,7 +2999,7 @@
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D21" s="37" t="s">
@@ -2995,22 +3009,22 @@
         <v>91</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G21" s="37" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I21" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J21" s="37" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="K21" s="37" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="L21" s="37">
         <v>2</v>
@@ -3022,8 +3036,8 @@
       <c r="N21" s="37">
         <v>100</v>
       </c>
-      <c r="O21" s="60" t="s">
-        <v>347</v>
+      <c r="O21" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P21" s="38">
         <v>4.4999999999999997E-3</v>
@@ -3041,7 +3055,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="C22" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="44" t="s">
@@ -3051,22 +3065,22 @@
         <v>92</v>
       </c>
       <c r="F22" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G22" s="44" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H22" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I22" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J22" s="44" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="K22" s="44" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="L22" s="44">
         <v>1</v>
@@ -3078,8 +3092,8 @@
       <c r="N22" s="44">
         <v>100</v>
       </c>
-      <c r="O22" s="61" t="s">
-        <v>347</v>
+      <c r="O22" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P22" s="45">
         <v>3.2000000000000002E-3</v>
@@ -3097,7 +3111,7 @@
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="50" t="s">
         <v>10</v>
       </c>
       <c r="D23" s="37" t="s">
@@ -3107,22 +3121,22 @@
         <v>93</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G23" s="37" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H23" s="37" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I23" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J23" s="37" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="K23" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L23" s="37">
         <v>1</v>
@@ -3134,8 +3148,8 @@
       <c r="N23" s="37">
         <v>10</v>
       </c>
-      <c r="O23" s="60" t="s">
-        <v>347</v>
+      <c r="O23" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P23" s="38">
         <v>6.6000000000000003E-2</v>
@@ -3153,7 +3167,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="50" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="44" t="s">
@@ -3163,22 +3177,22 @@
         <v>94</v>
       </c>
       <c r="F24" s="44" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G24" s="44" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H24" s="44" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I24" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J24" s="44" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="K24" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L24" s="44">
         <v>1</v>
@@ -3190,8 +3204,8 @@
       <c r="N24" s="44">
         <v>10</v>
       </c>
-      <c r="O24" s="61" t="s">
-        <v>347</v>
+      <c r="O24" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P24" s="45">
         <v>8.6400000000000005E-2</v>
@@ -3209,7 +3223,7 @@
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="50" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="37" t="s">
@@ -3219,22 +3233,22 @@
         <v>95</v>
       </c>
       <c r="F25" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G25" s="37" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H25" s="37" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I25" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J25" s="37" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="K25" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L25" s="37">
         <v>1</v>
@@ -3246,8 +3260,8 @@
       <c r="N25" s="37">
         <v>20</v>
       </c>
-      <c r="O25" s="60" t="s">
-        <v>347</v>
+      <c r="O25" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P25" s="38">
         <v>2.63E-2</v>
@@ -3265,7 +3279,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="59" t="s">
+      <c r="C26" s="51" t="s">
         <v>11</v>
       </c>
       <c r="D26" s="44" t="s">
@@ -3275,22 +3289,22 @@
         <v>96</v>
       </c>
       <c r="F26" s="44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G26" s="44" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H26" s="44" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I26" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J26" s="44" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="K26" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L26" s="44">
         <v>1</v>
@@ -3302,8 +3316,8 @@
       <c r="N26" s="44">
         <v>10</v>
       </c>
-      <c r="O26" s="61" t="s">
-        <v>347</v>
+      <c r="O26" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P26" s="45">
         <v>9.8199999999999996E-2</v>
@@ -3321,7 +3335,7 @@
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="50" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="37" t="s">
@@ -3331,22 +3345,22 @@
         <v>97</v>
       </c>
       <c r="F27" s="37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G27" s="37" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H27" s="37" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I27" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J27" s="37" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="K27" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L27" s="37">
         <v>2</v>
@@ -3358,8 +3372,8 @@
       <c r="N27" s="37">
         <v>20</v>
       </c>
-      <c r="O27" s="60" t="s">
-        <v>347</v>
+      <c r="O27" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P27" s="38">
         <v>3.2199999999999999E-2</v>
@@ -3377,7 +3391,7 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="59" t="s">
+      <c r="C28" s="51" t="s">
         <v>13</v>
       </c>
       <c r="D28" s="44" t="s">
@@ -3387,22 +3401,22 @@
         <v>98</v>
       </c>
       <c r="F28" s="44" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G28" s="44" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H28" s="44" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I28" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J28" s="44" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="K28" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L28" s="44">
         <v>1</v>
@@ -3414,8 +3428,8 @@
       <c r="N28" s="44">
         <v>50</v>
       </c>
-      <c r="O28" s="61" t="s">
-        <v>347</v>
+      <c r="O28" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P28" s="45">
         <v>8.8999999999999999E-3</v>
@@ -3433,7 +3447,7 @@
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="50" t="s">
         <v>14</v>
       </c>
       <c r="D29" s="37" t="s">
@@ -3443,22 +3457,22 @@
         <v>99</v>
       </c>
       <c r="F29" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G29" s="37" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H29" s="37" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I29" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J29" s="37" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="K29" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L29" s="37">
         <v>1</v>
@@ -3470,8 +3484,8 @@
       <c r="N29" s="37">
         <v>10</v>
       </c>
-      <c r="O29" s="60" t="s">
-        <v>347</v>
+      <c r="O29" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P29" s="38">
         <v>0.2213</v>
@@ -3489,7 +3503,7 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="59" t="s">
+      <c r="C30" s="51" t="s">
         <v>15</v>
       </c>
       <c r="D30" s="44" t="s">
@@ -3499,22 +3513,22 @@
         <v>100</v>
       </c>
       <c r="F30" s="44" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G30" s="44" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H30" s="44" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I30" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J30" s="44" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="K30" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L30" s="44">
         <v>2</v>
@@ -3526,8 +3540,8 @@
       <c r="N30" s="44">
         <v>20</v>
       </c>
-      <c r="O30" s="61" t="s">
-        <v>347</v>
+      <c r="O30" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P30" s="45">
         <v>3.39E-2</v>
@@ -3545,7 +3559,7 @@
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="58" t="s">
+      <c r="C31" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D31" s="37" t="s">
@@ -3555,22 +3569,22 @@
         <v>101</v>
       </c>
       <c r="F31" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H31" s="37" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I31" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J31" s="37" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="K31" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L31" s="37">
         <v>1</v>
@@ -3582,8 +3596,8 @@
       <c r="N31" s="37">
         <v>6</v>
       </c>
-      <c r="O31" s="60" t="s">
-        <v>347</v>
+      <c r="O31" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P31" s="38">
         <v>1.4796</v>
@@ -3601,7 +3615,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="59"/>
+      <c r="C32" s="51"/>
       <c r="D32" s="44" t="s">
         <v>45</v>
       </c>
@@ -3609,22 +3623,22 @@
         <v>102</v>
       </c>
       <c r="F32" s="44" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G32" s="44" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H32" s="44" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I32" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J32" s="44" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="K32" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L32" s="44">
         <v>1</v>
@@ -3636,8 +3650,8 @@
       <c r="N32" s="44">
         <v>6</v>
       </c>
-      <c r="O32" s="61" t="s">
-        <v>347</v>
+      <c r="O32" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P32" s="45">
         <v>0.9546</v>
@@ -3655,7 +3669,7 @@
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="58" t="s">
+      <c r="C33" s="50" t="s">
         <v>15</v>
       </c>
       <c r="D33" s="37" t="s">
@@ -3665,22 +3679,22 @@
         <v>103</v>
       </c>
       <c r="F33" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G33" s="37" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H33" s="37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I33" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J33" s="37" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="K33" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L33" s="37">
         <v>1</v>
@@ -3692,8 +3706,8 @@
       <c r="N33" s="37">
         <v>10</v>
       </c>
-      <c r="O33" s="60" t="s">
-        <v>347</v>
+      <c r="O33" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P33" s="38">
         <v>4.1300000000000003E-2</v>
@@ -3711,7 +3725,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="59" t="s">
+      <c r="C34" s="51" t="s">
         <v>13</v>
       </c>
       <c r="D34" s="44" t="s">
@@ -3721,22 +3735,22 @@
         <v>104</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G34" s="44" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H34" s="44" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I34" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J34" s="44" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="K34" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L34" s="44">
         <v>1</v>
@@ -3748,8 +3762,8 @@
       <c r="N34" s="44">
         <v>6</v>
       </c>
-      <c r="O34" s="61" t="s">
-        <v>347</v>
+      <c r="O34" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P34" s="45">
         <v>0.29110000000000003</v>
@@ -3767,54 +3781,54 @@
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="58" t="s">
+      <c r="C35" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="D35" s="62" t="s">
+      <c r="D35" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="62" t="s">
+      <c r="E35" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="F35" s="62" t="s">
-        <v>334</v>
-      </c>
-      <c r="G35" s="62" t="s">
-        <v>335</v>
-      </c>
-      <c r="H35" s="63" t="s">
-        <v>333</v>
-      </c>
-      <c r="I35" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="J35" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="K35" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="L35" s="62">
+      <c r="F35" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="G35" s="54" t="s">
+        <v>330</v>
+      </c>
+      <c r="H35" s="55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="J35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="K35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="L35" s="54">
         <v>13</v>
       </c>
-      <c r="M35" s="62">
+      <c r="M35" s="54">
         <f>L35*5</f>
         <v>65</v>
       </c>
-      <c r="N35" s="62" t="s">
-        <v>333</v>
-      </c>
-      <c r="O35" s="62" t="s">
-        <v>333</v>
-      </c>
-      <c r="P35" s="65" t="s">
-        <v>333</v>
-      </c>
-      <c r="Q35" s="65" t="s">
-        <v>333</v>
-      </c>
-      <c r="R35" s="62"/>
-      <c r="S35" s="66"/>
+      <c r="N35" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="O35" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="P35" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q35" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="R35" s="54"/>
+      <c r="S35" s="58"/>
     </row>
     <row r="36" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
@@ -3822,7 +3836,7 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="59" t="s">
+      <c r="C36" s="51" t="s">
         <v>18</v>
       </c>
       <c r="D36" s="44" t="s">
@@ -3832,22 +3846,22 @@
         <v>106</v>
       </c>
       <c r="F36" s="44" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G36" s="44" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H36" s="44" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I36" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J36" s="44" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="K36" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L36" s="44">
         <v>1</v>
@@ -3859,8 +3873,8 @@
       <c r="N36" s="44">
         <v>10</v>
       </c>
-      <c r="O36" s="61" t="s">
-        <v>347</v>
+      <c r="O36" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P36" s="45">
         <v>4.6899999999999997E-2</v>
@@ -3878,7 +3892,7 @@
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="59" t="s">
+      <c r="C37" s="51" t="s">
         <v>18</v>
       </c>
       <c r="D37" s="37" t="s">
@@ -3888,22 +3902,22 @@
         <v>107</v>
       </c>
       <c r="F37" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H37" s="37" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I37" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J37" s="37" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="K37" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L37" s="37">
         <v>1</v>
@@ -3915,8 +3929,8 @@
       <c r="N37" s="37">
         <v>20</v>
       </c>
-      <c r="O37" s="60" t="s">
-        <v>347</v>
+      <c r="O37" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P37" s="38">
         <v>3.49E-2</v>
@@ -3934,45 +3948,45 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="58" t="s">
+      <c r="C38" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D38" s="44" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E38" s="44" t="s">
         <v>108</v>
       </c>
       <c r="F38" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G38" s="44" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H38" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I38" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J38" s="44" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="K38" s="44" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="L38" s="44">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M38" s="44">
         <f t="shared" ref="M38" si="29">L38*5</f>
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="N38" s="44">
         <v>100</v>
       </c>
-      <c r="O38" s="61" t="s">
-        <v>347</v>
+      <c r="O38" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P38" s="45">
         <v>1E-3</v>
@@ -3990,7 +4004,7 @@
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="58" t="s">
+      <c r="C39" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D39" s="37" t="s">
@@ -4000,22 +4014,22 @@
         <v>109</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I39" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J39" s="37" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="K39" s="37" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="L39" s="37">
         <v>3</v>
@@ -4027,8 +4041,8 @@
       <c r="N39" s="37">
         <v>100</v>
       </c>
-      <c r="O39" s="60" t="s">
-        <v>347</v>
+      <c r="O39" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P39" s="38">
         <v>1.1999999999999999E-3</v>
@@ -4046,7 +4060,7 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="58" t="s">
+      <c r="C40" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D40" s="44" t="s">
@@ -4056,22 +4070,22 @@
         <v>110</v>
       </c>
       <c r="F40" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G40" s="44" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H40" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I40" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J40" s="44" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="K40" s="44" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="L40" s="44">
         <v>3</v>
@@ -4083,8 +4097,8 @@
       <c r="N40" s="44">
         <v>100</v>
       </c>
-      <c r="O40" s="61" t="s">
-        <v>347</v>
+      <c r="O40" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P40" s="45">
         <v>1.1000000000000001E-3</v>
@@ -4102,7 +4116,7 @@
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="58" t="s">
+      <c r="C41" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D41" s="37" t="s">
@@ -4112,22 +4126,22 @@
         <v>111</v>
       </c>
       <c r="F41" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G41" s="37" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H41" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I41" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J41" s="37" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="K41" s="37" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="L41" s="37">
         <v>1</v>
@@ -4139,8 +4153,8 @@
       <c r="N41" s="37">
         <v>100</v>
       </c>
-      <c r="O41" s="60" t="s">
-        <v>347</v>
+      <c r="O41" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P41" s="38">
         <v>1.1999999999999999E-3</v>
@@ -4158,7 +4172,7 @@
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="58" t="s">
+      <c r="C42" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D42" s="37" t="s">
@@ -4168,22 +4182,22 @@
         <v>112</v>
       </c>
       <c r="F42" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G42" s="37" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H42" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J42" s="37" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="K42" s="37" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="L42" s="37">
         <v>2</v>
@@ -4195,8 +4209,8 @@
       <c r="N42" s="37">
         <v>100</v>
       </c>
-      <c r="O42" s="60" t="s">
-        <v>347</v>
+      <c r="O42" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P42" s="38">
         <v>1.1000000000000001E-3</v>
@@ -4208,36 +4222,38 @@
       <c r="R42" s="37"/>
       <c r="S42" s="49"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="40">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="58" t="s">
+      <c r="C43" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D43" s="44" t="s">
         <v>55</v>
       </c>
       <c r="E43" s="44" t="s">
-        <v>113</v>
+        <v>353</v>
       </c>
       <c r="F43" s="44" t="s">
-        <v>154</v>
+        <v>350</v>
       </c>
       <c r="G43" s="44" t="s">
-        <v>199</v>
+        <v>351</v>
       </c>
       <c r="H43" s="44" t="s">
-        <v>222</v>
-      </c>
-      <c r="I43" s="44"/>
+        <v>219</v>
+      </c>
+      <c r="I43" s="44" t="s">
+        <v>328</v>
+      </c>
       <c r="J43" s="44" t="s">
-        <v>280</v>
+        <v>352</v>
       </c>
       <c r="K43" s="44" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="L43" s="44">
         <v>1</v>
@@ -4246,12 +4262,18 @@
         <f t="shared" ref="M43" si="33">L43*5</f>
         <v>5</v>
       </c>
-      <c r="N43" s="44"/>
-      <c r="O43" s="44"/>
-      <c r="P43" s="45"/>
+      <c r="N43" s="44">
+        <v>20</v>
+      </c>
+      <c r="O43" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="P43" s="45">
+        <v>2.7699999999999999E-2</v>
+      </c>
       <c r="Q43" s="45">
         <f t="shared" ref="Q43" si="34">P43*N43</f>
-        <v>0</v>
+        <v>0.55399999999999994</v>
       </c>
       <c r="R43" s="44"/>
       <c r="S43" s="49"/>
@@ -4262,32 +4284,32 @@
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="58" t="s">
+      <c r="C44" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D44" s="37" t="s">
         <v>56</v>
       </c>
       <c r="E44" s="37" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F44" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G44" s="37" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H44" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J44" s="37" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="K44" s="37" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="L44" s="37">
         <v>5</v>
@@ -4299,8 +4321,8 @@
       <c r="N44" s="37">
         <v>100</v>
       </c>
-      <c r="O44" s="60" t="s">
-        <v>347</v>
+      <c r="O44" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P44" s="38">
         <v>1.1999999999999999E-3</v>
@@ -4318,32 +4340,32 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="58" t="s">
+      <c r="C45" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D45" s="44" t="s">
         <v>57</v>
       </c>
       <c r="E45" s="44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F45" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G45" s="44" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H45" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J45" s="44" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="K45" s="44" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="L45" s="44">
         <v>2</v>
@@ -4355,8 +4377,8 @@
       <c r="N45" s="44">
         <v>100</v>
       </c>
-      <c r="O45" s="61" t="s">
-        <v>347</v>
+      <c r="O45" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P45" s="45">
         <v>3.0999999999999999E-3</v>
@@ -4374,32 +4396,32 @@
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="58" t="s">
+      <c r="C46" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D46" s="37" t="s">
         <v>58</v>
       </c>
       <c r="E46" s="37" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F46" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G46" s="37" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H46" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I46" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J46" s="37" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="K46" s="37" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="L46" s="37">
         <v>3</v>
@@ -4411,8 +4433,8 @@
       <c r="N46" s="37">
         <v>100</v>
       </c>
-      <c r="O46" s="60" t="s">
-        <v>347</v>
+      <c r="O46" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P46" s="38">
         <v>1.1000000000000001E-3</v>
@@ -4430,32 +4452,32 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="58" t="s">
+      <c r="C47" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D47" s="44" t="s">
         <v>59</v>
       </c>
       <c r="E47" s="44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F47" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G47" s="44" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H47" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I47" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J47" s="44" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="K47" s="44" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="L47" s="44">
         <v>2</v>
@@ -4467,8 +4489,8 @@
       <c r="N47" s="44">
         <v>100</v>
       </c>
-      <c r="O47" s="61" t="s">
-        <v>347</v>
+      <c r="O47" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P47" s="45">
         <v>1.1999999999999999E-3</v>
@@ -4486,32 +4508,32 @@
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="58" t="s">
+      <c r="C48" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D48" s="37" t="s">
         <v>60</v>
       </c>
       <c r="E48" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F48" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G48" s="37" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H48" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I48" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J48" s="37" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="K48" s="37" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="L48" s="37">
         <v>2</v>
@@ -4523,8 +4545,8 @@
       <c r="N48" s="37">
         <v>100</v>
       </c>
-      <c r="O48" s="60" t="s">
-        <v>347</v>
+      <c r="O48" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P48" s="38">
         <v>1.8E-3</v>
@@ -4542,32 +4564,32 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="58" t="s">
+      <c r="C49" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D49" s="44" t="s">
         <v>61</v>
       </c>
       <c r="E49" s="44" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F49" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G49" s="44" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H49" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I49" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J49" s="44" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="K49" s="44" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="L49" s="44">
         <v>1</v>
@@ -4579,8 +4601,8 @@
       <c r="N49" s="44">
         <v>20</v>
       </c>
-      <c r="O49" s="61" t="s">
-        <v>347</v>
+      <c r="O49" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P49" s="45">
         <v>2.75E-2</v>
@@ -4598,32 +4620,32 @@
         <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
-      <c r="C50" s="58" t="s">
+      <c r="C50" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D50" s="37" t="s">
         <v>62</v>
       </c>
       <c r="E50" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F50" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G50" s="37" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H50" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I50" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J50" s="37" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="K50" s="37" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="L50" s="37">
         <v>1</v>
@@ -4635,8 +4657,8 @@
       <c r="N50" s="37">
         <v>50</v>
       </c>
-      <c r="O50" s="60" t="s">
-        <v>347</v>
+      <c r="O50" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P50" s="38">
         <v>8.8000000000000005E-3</v>
@@ -4654,32 +4676,32 @@
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="58" t="s">
+      <c r="C51" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D51" s="44" t="s">
         <v>63</v>
       </c>
       <c r="E51" s="44" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F51" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G51" s="44" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H51" s="44" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I51" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J51" s="44" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="K51" s="44" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="L51" s="44">
         <v>1</v>
@@ -4691,8 +4713,8 @@
       <c r="N51" s="44">
         <v>20</v>
       </c>
-      <c r="O51" s="61" t="s">
-        <v>347</v>
+      <c r="O51" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P51" s="45">
         <v>2.63E-2</v>
@@ -4710,32 +4732,32 @@
         <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
-      <c r="C52" s="58" t="s">
+      <c r="C52" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D52" s="37" t="s">
         <v>64</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G52" s="37" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H52" s="37" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I52" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J52" s="37" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="K52" s="37" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="L52" s="37">
         <v>1</v>
@@ -4747,8 +4769,8 @@
       <c r="N52" s="37">
         <v>20</v>
       </c>
-      <c r="O52" s="60" t="s">
-        <v>347</v>
+      <c r="O52" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P52" s="38">
         <v>3.1E-2</v>
@@ -4766,32 +4788,32 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C53" s="58" t="s">
+      <c r="C53" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D53" s="44" t="s">
         <v>65</v>
       </c>
       <c r="E53" s="44" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F53" s="44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G53" s="44" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H53" s="44" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I53" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J53" s="44" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="K53" s="44" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="L53" s="44">
         <v>1</v>
@@ -4803,8 +4825,8 @@
       <c r="N53" s="44">
         <v>100</v>
       </c>
-      <c r="O53" s="61" t="s">
-        <v>347</v>
+      <c r="O53" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P53" s="45">
         <v>1.1999999999999999E-3</v>
@@ -4822,54 +4844,54 @@
         <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
-      <c r="C54" s="58" t="s">
-        <v>155</v>
-      </c>
-      <c r="D54" s="62" t="s">
+      <c r="C54" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="D54" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="E54" s="62" t="s">
-        <v>124</v>
-      </c>
-      <c r="F54" s="62" t="s">
-        <v>334</v>
-      </c>
-      <c r="G54" s="62" t="s">
-        <v>155</v>
-      </c>
-      <c r="H54" s="63" t="s">
-        <v>333</v>
-      </c>
-      <c r="I54" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="J54" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="K54" s="62" t="s">
-        <v>333</v>
-      </c>
-      <c r="L54" s="62">
+      <c r="E54" s="54" t="s">
+        <v>123</v>
+      </c>
+      <c r="F54" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="G54" s="54" t="s">
+        <v>153</v>
+      </c>
+      <c r="H54" s="55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="J54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="K54" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="L54" s="54">
         <v>3</v>
       </c>
-      <c r="M54" s="62">
+      <c r="M54" s="54">
         <f>L54*5</f>
         <v>15</v>
       </c>
-      <c r="N54" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="O54" s="64" t="s">
-        <v>333</v>
-      </c>
-      <c r="P54" s="65" t="s">
-        <v>333</v>
-      </c>
-      <c r="Q54" s="65" t="s">
-        <v>333</v>
-      </c>
-      <c r="R54" s="62"/>
-      <c r="S54" s="66"/>
+      <c r="N54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="O54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="P54" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q54" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="R54" s="54"/>
+      <c r="S54" s="58"/>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
@@ -4877,32 +4899,32 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C55" s="59" t="s">
+      <c r="C55" s="51" t="s">
         <v>20</v>
       </c>
       <c r="D55" s="44" t="s">
         <v>67</v>
       </c>
       <c r="E55" s="44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F55" s="44" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G55" s="44" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H55" s="44" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I55" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J55" s="44" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="K55" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L55" s="44">
         <v>5</v>
@@ -4914,8 +4936,8 @@
       <c r="N55" s="44">
         <v>30</v>
       </c>
-      <c r="O55" s="61" t="s">
-        <v>347</v>
+      <c r="O55" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P55" s="45">
         <v>0.3135</v>
@@ -4933,32 +4955,32 @@
         <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
-      <c r="C56" s="59" t="s">
+      <c r="C56" s="51" t="s">
         <v>20</v>
       </c>
       <c r="D56" s="44" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="E56" s="44" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F56" s="44" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G56" s="44" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H56" s="44" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I56" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J56" s="44" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="K56" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L56" s="44">
         <v>1</v>
@@ -4970,8 +4992,8 @@
       <c r="N56" s="44">
         <v>10</v>
       </c>
-      <c r="O56" s="61" t="s">
-        <v>347</v>
+      <c r="O56" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P56" s="45">
         <v>6.2100000000000002E-2</v>
@@ -4989,32 +5011,32 @@
         <f>ROW(B57) - ROW($B$9)</f>
         <v>48</v>
       </c>
-      <c r="C57" s="58" t="s">
+      <c r="C57" s="50" t="s">
         <v>21</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>68</v>
       </c>
       <c r="E57" s="37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F57" s="37" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G57" s="37" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H57" s="37" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I57" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J57" s="37" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="K57" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L57" s="37">
         <v>1</v>
@@ -5026,8 +5048,8 @@
       <c r="N57" s="37">
         <v>6</v>
       </c>
-      <c r="O57" s="60" t="s">
-        <v>347</v>
+      <c r="O57" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P57" s="38">
         <v>0.16209999999999999</v>
@@ -5045,28 +5067,32 @@
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="C58" s="59" t="s">
+      <c r="C58" s="51" t="s">
         <v>21</v>
       </c>
       <c r="D58" s="44" t="s">
         <v>69</v>
       </c>
       <c r="E58" s="44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F58" s="44" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G58" s="44" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H58" s="44" t="s">
-        <v>239</v>
-      </c>
-      <c r="I58" s="44"/>
-      <c r="J58" s="44"/>
+        <v>236</v>
+      </c>
+      <c r="I58" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J58" s="44" t="s">
+        <v>348</v>
+      </c>
       <c r="K58" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L58" s="44">
         <v>1</v>
@@ -5075,12 +5101,18 @@
         <f t="shared" ref="M58" si="49">L58*5</f>
         <v>5</v>
       </c>
-      <c r="N58" s="44"/>
-      <c r="O58" s="44"/>
-      <c r="P58" s="45"/>
+      <c r="N58" s="44">
+        <v>10</v>
+      </c>
+      <c r="O58" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="P58" s="45">
+        <v>0.1341</v>
+      </c>
       <c r="Q58" s="45">
         <f t="shared" ref="Q58" si="50">P58*N58</f>
-        <v>0</v>
+        <v>1.341</v>
       </c>
       <c r="R58" s="44"/>
       <c r="S58" s="49"/>
@@ -5091,32 +5123,32 @@
         <f>ROW(B59) - ROW($B$9)</f>
         <v>50</v>
       </c>
-      <c r="C59" s="58" t="s">
+      <c r="C59" s="50" t="s">
         <v>18</v>
       </c>
       <c r="D59" s="37" t="s">
         <v>70</v>
       </c>
       <c r="E59" s="37" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F59" s="37" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G59" s="37" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H59" s="37" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="I59" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J59" s="37" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="K59" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L59" s="37">
         <v>1</v>
@@ -5128,8 +5160,8 @@
       <c r="N59" s="37">
         <v>10</v>
       </c>
-      <c r="O59" s="60" t="s">
-        <v>347</v>
+      <c r="O59" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P59" s="38">
         <v>0.19539999999999999</v>
@@ -5147,32 +5179,32 @@
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="C60" s="59" t="s">
+      <c r="C60" s="51" t="s">
         <v>21</v>
       </c>
       <c r="D60" s="44" t="s">
         <v>71</v>
       </c>
       <c r="E60" s="44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F60" s="44" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G60" s="44" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H60" s="44" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I60" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J60" s="44" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="K60" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L60" s="44">
         <v>1</v>
@@ -5184,8 +5216,8 @@
       <c r="N60" s="44">
         <v>6</v>
       </c>
-      <c r="O60" s="61" t="s">
-        <v>347</v>
+      <c r="O60" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P60" s="45">
         <v>0.43909999999999999</v>
@@ -5203,32 +5235,32 @@
         <f>ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
-      <c r="C61" s="58" t="s">
+      <c r="C61" s="50" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="37" t="s">
         <v>72</v>
       </c>
       <c r="E61" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F61" s="37" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G61" s="37" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H61" s="37" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I61" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J61" s="37" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="K61" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L61" s="37">
         <v>1</v>
@@ -5240,8 +5272,8 @@
       <c r="N61" s="37">
         <v>10</v>
       </c>
-      <c r="O61" s="60" t="s">
-        <v>347</v>
+      <c r="O61" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P61" s="38">
         <v>0.15479999999999999</v>
@@ -5259,32 +5291,32 @@
         <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
-      <c r="C62" s="58" t="s">
+      <c r="C62" s="50" t="s">
         <v>22</v>
       </c>
       <c r="D62" s="37" t="s">
         <v>73</v>
       </c>
       <c r="E62" s="37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F62" s="37" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G62" s="37" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H62" s="37" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="I62" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J62" s="37" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="K62" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L62" s="37">
         <v>1</v>
@@ -5296,8 +5328,8 @@
       <c r="N62" s="37">
         <v>6</v>
       </c>
-      <c r="O62" s="60" t="s">
-        <v>347</v>
+      <c r="O62" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P62" s="38">
         <v>5.1212</v>
@@ -5315,32 +5347,32 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C63" s="59" t="s">
+      <c r="C63" s="51" t="s">
         <v>21</v>
       </c>
       <c r="D63" s="44" t="s">
         <v>74</v>
       </c>
       <c r="E63" s="44" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F63" s="44" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G63" s="44" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H63" s="44" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="I63" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J63" s="44" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="K63" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L63" s="44">
         <v>1</v>
@@ -5352,8 +5384,8 @@
       <c r="N63" s="44">
         <v>10</v>
       </c>
-      <c r="O63" s="61" t="s">
-        <v>347</v>
+      <c r="O63" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P63" s="45">
         <v>0.15670000000000001</v>
@@ -5371,32 +5403,32 @@
         <f>ROW(B64) - ROW($B$9)</f>
         <v>55</v>
       </c>
-      <c r="C64" s="58" t="s">
+      <c r="C64" s="50" t="s">
         <v>21</v>
       </c>
       <c r="D64" s="37" t="s">
         <v>75</v>
       </c>
       <c r="E64" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F64" s="37" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G64" s="37" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H64" s="37" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="I64" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J64" s="37" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="K64" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L64" s="37">
         <v>1</v>
@@ -5408,8 +5440,8 @@
       <c r="N64" s="37">
         <v>6</v>
       </c>
-      <c r="O64" s="60" t="s">
-        <v>347</v>
+      <c r="O64" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P64" s="38">
         <v>0.96889999999999998</v>
@@ -5427,32 +5459,32 @@
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C65" s="59" t="s">
+      <c r="C65" s="51" t="s">
         <v>21</v>
       </c>
       <c r="D65" s="44" t="s">
         <v>76</v>
       </c>
       <c r="E65" s="44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F65" s="44" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G65" s="44" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H65" s="44" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="I65" s="44" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J65" s="44" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="K65" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L65" s="44">
         <v>1</v>
@@ -5464,8 +5496,8 @@
       <c r="N65" s="44">
         <v>6</v>
       </c>
-      <c r="O65" s="61" t="s">
-        <v>347</v>
+      <c r="O65" s="53" t="s">
+        <v>342</v>
       </c>
       <c r="P65" s="45">
         <v>0.28870000000000001</v>
@@ -5483,32 +5515,32 @@
         <f>ROW(B66) - ROW($B$9)</f>
         <v>57</v>
       </c>
-      <c r="C66" s="58" t="s">
+      <c r="C66" s="50" t="s">
         <v>21</v>
       </c>
       <c r="D66" s="37" t="s">
         <v>77</v>
       </c>
       <c r="E66" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F66" s="37" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G66" s="37" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H66" s="37" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I66" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J66" s="37" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="K66" s="37" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="L66" s="37">
         <v>1</v>
@@ -5520,8 +5552,8 @@
       <c r="N66" s="37">
         <v>6</v>
       </c>
-      <c r="O66" s="60" t="s">
-        <v>347</v>
+      <c r="O66" s="52" t="s">
+        <v>342</v>
       </c>
       <c r="P66" s="38">
         <v>2.0651000000000002</v>
@@ -5535,36 +5567,36 @@
     </row>
     <row r="67" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
-      <c r="B67" s="67">
+      <c r="B67" s="59">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C67" s="68" t="s">
+      <c r="C67" s="60" t="s">
         <v>21</v>
       </c>
       <c r="D67" s="49" t="s">
         <v>78</v>
       </c>
       <c r="E67" s="49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F67" s="49" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G67" s="49" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H67" s="49" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="I67" s="49" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="J67" s="49" t="s">
-        <v>302</v>
-      </c>
-      <c r="K67" s="69" t="s">
-        <v>333</v>
+        <v>297</v>
+      </c>
+      <c r="K67" s="61" t="s">
+        <v>328</v>
       </c>
       <c r="L67" s="49">
         <v>1</v>
@@ -5576,13 +5608,13 @@
       <c r="N67" s="49">
         <v>6</v>
       </c>
-      <c r="O67" s="70" t="s">
-        <v>347</v>
-      </c>
-      <c r="P67" s="71">
+      <c r="O67" s="62" t="s">
+        <v>342</v>
+      </c>
+      <c r="P67" s="63">
         <v>1.2919</v>
       </c>
-      <c r="Q67" s="71">
+      <c r="Q67" s="63">
         <f t="shared" ref="Q67" si="58">P67*N67</f>
         <v>7.7514000000000003</v>
       </c>
@@ -5591,29 +5623,29 @@
     </row>
     <row r="68" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
-      <c r="B68" s="72"/>
-      <c r="C68" s="73"/>
-      <c r="D68" s="74"/>
-      <c r="E68" s="75"/>
-      <c r="F68" s="76"/>
-      <c r="G68" s="77"/>
-      <c r="H68" s="76"/>
-      <c r="I68" s="77"/>
-      <c r="J68" s="76"/>
-      <c r="K68" s="77"/>
-      <c r="L68" s="77"/>
-      <c r="M68" s="77"/>
-      <c r="N68" s="56" t="s">
+      <c r="B68" s="64"/>
+      <c r="C68" s="65"/>
+      <c r="D68" s="66"/>
+      <c r="E68" s="67"/>
+      <c r="F68" s="68"/>
+      <c r="G68" s="69"/>
+      <c r="H68" s="68"/>
+      <c r="I68" s="69"/>
+      <c r="J68" s="68"/>
+      <c r="K68" s="69"/>
+      <c r="L68" s="69"/>
+      <c r="M68" s="69"/>
+      <c r="N68" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="O68" s="57"/>
-      <c r="P68" s="57"/>
+      <c r="O68" s="79"/>
+      <c r="P68" s="79"/>
       <c r="Q68" s="41">
         <f>SUM(Q10:Q67)</f>
-        <v>132.43659999999997</v>
-      </c>
-      <c r="R68" s="78"/>
-      <c r="S68" s="79"/>
+        <v>134.60659999999996</v>
+      </c>
+      <c r="R68" s="74"/>
+      <c r="S68" s="75"/>
     </row>
     <row r="69" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -5629,17 +5661,17 @@
       <c r="K69" s="10"/>
       <c r="L69" s="10"/>
       <c r="M69" s="10"/>
-      <c r="N69" s="56" t="s">
+      <c r="N69" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="O69" s="57"/>
-      <c r="P69" s="57"/>
+      <c r="O69" s="79"/>
+      <c r="P69" s="79"/>
       <c r="Q69" s="42">
         <f>Q68/5</f>
-        <v>26.487319999999993</v>
-      </c>
-      <c r="R69" s="54"/>
-      <c r="S69" s="55"/>
+        <v>26.921319999999991</v>
+      </c>
+      <c r="R69" s="76"/>
+      <c r="S69" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5703,9 +5735,12 @@
     <hyperlink ref="O65" r:id="rId51"/>
     <hyperlink ref="O66" r:id="rId52"/>
     <hyperlink ref="O67" r:id="rId53"/>
+    <hyperlink ref="O18" r:id="rId54"/>
+    <hyperlink ref="O58" r:id="rId55"/>
+    <hyperlink ref="O43" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId54"/>
-  <drawing r:id="rId55"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId57"/>
+  <drawing r:id="rId58"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#6 eSpark BOM and JLCPCB BOM Completed
</commit_message>
<xml_diff>
--- a/BOM/eSpark-BOM.xlsx
+++ b/BOM/eSpark-BOM.xlsx
@@ -12,14 +12,15 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="1 Board" sheetId="2" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="358">
   <si>
     <t>Component list</t>
   </si>
@@ -1081,6 +1082,18 @@
   </si>
   <si>
     <t>General Purpose Chip Resistor Thick Film 1206 5.6Ohm 1% Paper T/R</t>
+  </si>
+  <si>
+    <t>LCSC/MOQ</t>
+  </si>
+  <si>
+    <t>UnitCost (1 Boards)</t>
+  </si>
+  <si>
+    <t>TotalCost (1 Boards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R9 = DNP that’s why not added in BOM </t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1105,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1254,6 +1267,14 @@
     </font>
     <font>
       <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1548,7 +1569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1771,6 +1792,65 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1796,6 +1876,60 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20783550" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2112,8 +2246,3371 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R68"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.5703125" customWidth="1"/>
+    <col min="18" max="18" width="26.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="71"/>
+    </row>
+    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="3"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="72"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="73"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="73"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="73"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="73"/>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="73"/>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>332</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>331</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>326</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>354</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>335</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>338</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="80"/>
+      <c r="B10" s="39">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>345</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>247</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>298</v>
+      </c>
+      <c r="L10" s="37">
+        <v>3</v>
+      </c>
+      <c r="M10" s="37">
+        <v>50</v>
+      </c>
+      <c r="N10" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O10" s="38">
+        <v>1.89E-2</v>
+      </c>
+      <c r="P10" s="38">
+        <f>O10*M10</f>
+        <v>0.94500000000000006</v>
+      </c>
+      <c r="Q10" s="37"/>
+      <c r="R10" s="81"/>
+    </row>
+    <row r="11" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="80"/>
+      <c r="B11" s="40">
+        <f t="shared" ref="B11:B67" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="G11" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="H11" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="I11" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J11" s="44" t="s">
+        <v>248</v>
+      </c>
+      <c r="K11" s="44" t="s">
+        <v>299</v>
+      </c>
+      <c r="L11" s="44">
+        <v>2</v>
+      </c>
+      <c r="M11" s="44">
+        <v>3</v>
+      </c>
+      <c r="N11" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O11" s="45">
+        <v>1.4064000000000001</v>
+      </c>
+      <c r="P11" s="45">
+        <f t="shared" ref="P11" si="1">O11*M11</f>
+        <v>4.2192000000000007</v>
+      </c>
+      <c r="Q11" s="44"/>
+      <c r="R11" s="44"/>
+    </row>
+    <row r="12" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A12" s="80"/>
+      <c r="B12" s="39">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>300</v>
+      </c>
+      <c r="L12" s="37">
+        <v>14</v>
+      </c>
+      <c r="M12" s="37">
+        <v>100</v>
+      </c>
+      <c r="N12" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O12" s="38">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="P12" s="38">
+        <f>O12*M12</f>
+        <v>0.5</v>
+      </c>
+      <c r="Q12" s="37"/>
+      <c r="R12" s="49"/>
+    </row>
+    <row r="13" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="80"/>
+      <c r="B13" s="40">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G13" s="44" t="s">
+        <v>171</v>
+      </c>
+      <c r="H13" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I13" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J13" s="44" t="s">
+        <v>250</v>
+      </c>
+      <c r="K13" s="44" t="s">
+        <v>301</v>
+      </c>
+      <c r="L13" s="44">
+        <v>1</v>
+      </c>
+      <c r="M13" s="44">
+        <v>100</v>
+      </c>
+      <c r="N13" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O13" s="45">
+        <v>2.8E-3</v>
+      </c>
+      <c r="P13" s="45">
+        <f t="shared" ref="P13" si="2">O13*M13</f>
+        <v>0.27999999999999997</v>
+      </c>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="49"/>
+    </row>
+    <row r="14" spans="1:18" s="82" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A14" s="80"/>
+      <c r="B14" s="39">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>251</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="L14" s="37">
+        <v>25</v>
+      </c>
+      <c r="M14" s="37">
+        <v>100</v>
+      </c>
+      <c r="N14" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O14" s="38">
+        <v>1.8E-3</v>
+      </c>
+      <c r="P14" s="38">
+        <f>O14*M14</f>
+        <v>0.18</v>
+      </c>
+      <c r="Q14" s="37"/>
+      <c r="R14" s="49"/>
+    </row>
+    <row r="15" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="80"/>
+      <c r="B15" s="40">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G15" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="H15" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I15" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J15" s="44" t="s">
+        <v>252</v>
+      </c>
+      <c r="K15" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="L15" s="44">
+        <v>2</v>
+      </c>
+      <c r="M15" s="44">
+        <v>5</v>
+      </c>
+      <c r="N15" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O15" s="45">
+        <v>0.16370000000000001</v>
+      </c>
+      <c r="P15" s="45">
+        <f t="shared" ref="P15" si="3">O15*M15</f>
+        <v>0.81850000000000001</v>
+      </c>
+      <c r="Q15" s="44"/>
+      <c r="R15" s="49"/>
+    </row>
+    <row r="16" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="80"/>
+      <c r="B16" s="39">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>221</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="K16" s="37" t="s">
+        <v>304</v>
+      </c>
+      <c r="L16" s="37">
+        <v>2</v>
+      </c>
+      <c r="M16" s="37">
+        <v>5</v>
+      </c>
+      <c r="N16" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O16" s="38">
+        <v>0.42320000000000002</v>
+      </c>
+      <c r="P16" s="38">
+        <f>O16*M16</f>
+        <v>2.1160000000000001</v>
+      </c>
+      <c r="Q16" s="37"/>
+      <c r="R16" s="49"/>
+    </row>
+    <row r="17" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="80"/>
+      <c r="B17" s="40">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G17" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="H17" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I17" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J17" s="44" t="s">
+        <v>254</v>
+      </c>
+      <c r="K17" s="44" t="s">
+        <v>305</v>
+      </c>
+      <c r="L17" s="44">
+        <v>6</v>
+      </c>
+      <c r="M17" s="44">
+        <v>20</v>
+      </c>
+      <c r="N17" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O17" s="45">
+        <v>2.3800000000000002E-2</v>
+      </c>
+      <c r="P17" s="45">
+        <f t="shared" ref="P17" si="4">O17*M17</f>
+        <v>0.47600000000000003</v>
+      </c>
+      <c r="Q17" s="44"/>
+      <c r="R17" s="49"/>
+    </row>
+    <row r="18" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="80"/>
+      <c r="B18" s="39">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="G18" s="54" t="s">
+        <v>176</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>346</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>347</v>
+      </c>
+      <c r="K18" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="L18" s="37">
+        <v>3</v>
+      </c>
+      <c r="M18" s="37">
+        <v>50</v>
+      </c>
+      <c r="N18" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O18" s="38">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="P18" s="38">
+        <f>O18*M18</f>
+        <v>0.27499999999999997</v>
+      </c>
+      <c r="Q18" s="37"/>
+      <c r="R18" s="49"/>
+    </row>
+    <row r="19" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="80"/>
+      <c r="B19" s="40">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="44" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G19" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="H19" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I19" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J19" s="44" t="s">
+        <v>255</v>
+      </c>
+      <c r="K19" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="L19" s="44">
+        <v>1</v>
+      </c>
+      <c r="M19" s="44">
+        <v>20</v>
+      </c>
+      <c r="N19" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O19" s="45">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="P19" s="45">
+        <f t="shared" ref="P19:P20" si="5">O19*M19</f>
+        <v>0.40399999999999997</v>
+      </c>
+      <c r="Q19" s="44"/>
+      <c r="R19" s="49"/>
+    </row>
+    <row r="20" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="80"/>
+      <c r="B20" s="40">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="C20" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="44" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="44" t="s">
+        <v>178</v>
+      </c>
+      <c r="H20" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I20" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J20" s="44" t="s">
+        <v>256</v>
+      </c>
+      <c r="K20" s="44" t="s">
+        <v>307</v>
+      </c>
+      <c r="L20" s="44">
+        <v>2</v>
+      </c>
+      <c r="M20" s="44">
+        <v>100</v>
+      </c>
+      <c r="N20" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O20" s="45">
+        <v>3.7000000000000002E-3</v>
+      </c>
+      <c r="P20" s="45">
+        <f t="shared" si="5"/>
+        <v>0.37</v>
+      </c>
+      <c r="Q20" s="44"/>
+      <c r="R20" s="49"/>
+    </row>
+    <row r="21" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="80"/>
+      <c r="B21" s="39">
+        <f>ROW(B21) - ROW($B$9)</f>
+        <v>12</v>
+      </c>
+      <c r="C21" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="G21" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="H21" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J21" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="K21" s="37" t="s">
+        <v>308</v>
+      </c>
+      <c r="L21" s="37">
+        <v>2</v>
+      </c>
+      <c r="M21" s="37">
+        <v>100</v>
+      </c>
+      <c r="N21" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O21" s="38">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="P21" s="38">
+        <f>O21*M21</f>
+        <v>0.44999999999999996</v>
+      </c>
+      <c r="Q21" s="37"/>
+      <c r="R21" s="49"/>
+    </row>
+    <row r="22" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="80"/>
+      <c r="B22" s="40">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="C22" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="F22" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="G22" s="44" t="s">
+        <v>180</v>
+      </c>
+      <c r="H22" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I22" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J22" s="44" t="s">
+        <v>258</v>
+      </c>
+      <c r="K22" s="44" t="s">
+        <v>309</v>
+      </c>
+      <c r="L22" s="44">
+        <v>1</v>
+      </c>
+      <c r="M22" s="44">
+        <v>100</v>
+      </c>
+      <c r="N22" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O22" s="45">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="P22" s="45">
+        <f t="shared" ref="P22" si="6">O22*M22</f>
+        <v>0.32</v>
+      </c>
+      <c r="Q22" s="44"/>
+      <c r="R22" s="49"/>
+    </row>
+    <row r="23" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="80"/>
+      <c r="B23" s="39">
+        <f>ROW(B23) - ROW($B$9)</f>
+        <v>14</v>
+      </c>
+      <c r="C23" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="F23" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="G23" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="H23" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J23" s="37" t="s">
+        <v>259</v>
+      </c>
+      <c r="K23" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L23" s="37">
+        <v>1</v>
+      </c>
+      <c r="M23" s="37">
+        <v>10</v>
+      </c>
+      <c r="N23" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O23" s="38">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="P23" s="38">
+        <f>O23*M23</f>
+        <v>0.66</v>
+      </c>
+      <c r="Q23" s="37"/>
+      <c r="R23" s="49"/>
+    </row>
+    <row r="24" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A24" s="80"/>
+      <c r="B24" s="40">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="C24" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="44" t="s">
+        <v>143</v>
+      </c>
+      <c r="G24" s="44" t="s">
+        <v>182</v>
+      </c>
+      <c r="H24" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="I24" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J24" s="44" t="s">
+        <v>260</v>
+      </c>
+      <c r="K24" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L24" s="44">
+        <v>1</v>
+      </c>
+      <c r="M24" s="44">
+        <v>5</v>
+      </c>
+      <c r="N24" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O24" s="45">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="P24" s="45">
+        <f t="shared" ref="P24" si="7">O24*M24</f>
+        <v>0.43200000000000005</v>
+      </c>
+      <c r="Q24" s="44"/>
+      <c r="R24" s="49"/>
+    </row>
+    <row r="25" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A25" s="80"/>
+      <c r="B25" s="39">
+        <f>ROW(B25) - ROW($B$9)</f>
+        <v>16</v>
+      </c>
+      <c r="C25" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="G25" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="H25" s="37" t="s">
+        <v>225</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J25" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="K25" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L25" s="37">
+        <v>1</v>
+      </c>
+      <c r="M25" s="37">
+        <v>20</v>
+      </c>
+      <c r="N25" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O25" s="38">
+        <v>2.63E-2</v>
+      </c>
+      <c r="P25" s="38">
+        <f>O25*M25</f>
+        <v>0.52600000000000002</v>
+      </c>
+      <c r="Q25" s="37"/>
+      <c r="R25" s="49"/>
+    </row>
+    <row r="26" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A26" s="80"/>
+      <c r="B26" s="40">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C26" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" s="44" t="s">
+        <v>184</v>
+      </c>
+      <c r="H26" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="I26" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J26" s="44" t="s">
+        <v>262</v>
+      </c>
+      <c r="K26" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L26" s="44">
+        <v>1</v>
+      </c>
+      <c r="M26" s="44">
+        <v>5</v>
+      </c>
+      <c r="N26" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O26" s="45">
+        <v>9.8199999999999996E-2</v>
+      </c>
+      <c r="P26" s="45">
+        <f t="shared" ref="P26" si="8">O26*M26</f>
+        <v>0.49099999999999999</v>
+      </c>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="49"/>
+    </row>
+    <row r="27" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A27" s="80"/>
+      <c r="B27" s="39">
+        <f>ROW(B27) - ROW($B$9)</f>
+        <v>18</v>
+      </c>
+      <c r="C27" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="G27" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="H27" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J27" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="K27" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L27" s="37">
+        <v>2</v>
+      </c>
+      <c r="M27" s="37">
+        <v>20</v>
+      </c>
+      <c r="N27" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O27" s="38">
+        <v>3.2199999999999999E-2</v>
+      </c>
+      <c r="P27" s="38">
+        <f>O27*M27</f>
+        <v>0.64400000000000002</v>
+      </c>
+      <c r="Q27" s="37"/>
+      <c r="R27" s="49"/>
+    </row>
+    <row r="28" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A28" s="80"/>
+      <c r="B28" s="40">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="C28" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="F28" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="G28" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="H28" s="44" t="s">
+        <v>222</v>
+      </c>
+      <c r="I28" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J28" s="44" t="s">
+        <v>264</v>
+      </c>
+      <c r="K28" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L28" s="44">
+        <v>1</v>
+      </c>
+      <c r="M28" s="44">
+        <v>50</v>
+      </c>
+      <c r="N28" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O28" s="45">
+        <v>8.8999999999999999E-3</v>
+      </c>
+      <c r="P28" s="45">
+        <f t="shared" ref="P28" si="9">O28*M28</f>
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="Q28" s="44"/>
+      <c r="R28" s="49"/>
+    </row>
+    <row r="29" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A29" s="80"/>
+      <c r="B29" s="39">
+        <f>ROW(B29) - ROW($B$9)</f>
+        <v>20</v>
+      </c>
+      <c r="C29" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="37" t="s">
+        <v>329</v>
+      </c>
+      <c r="G29" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="H29" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J29" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="K29" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L29" s="37">
+        <v>1</v>
+      </c>
+      <c r="M29" s="37">
+        <v>5</v>
+      </c>
+      <c r="N29" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O29" s="38">
+        <v>0.2213</v>
+      </c>
+      <c r="P29" s="38">
+        <f>O29*M29</f>
+        <v>1.1065</v>
+      </c>
+      <c r="Q29" s="37"/>
+      <c r="R29" s="49"/>
+    </row>
+    <row r="30" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A30" s="80"/>
+      <c r="B30" s="40">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="C30" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="F30" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="G30" s="44" t="s">
+        <v>188</v>
+      </c>
+      <c r="H30" s="44" t="s">
+        <v>228</v>
+      </c>
+      <c r="I30" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J30" s="44" t="s">
+        <v>266</v>
+      </c>
+      <c r="K30" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L30" s="44">
+        <v>2</v>
+      </c>
+      <c r="M30" s="44">
+        <v>20</v>
+      </c>
+      <c r="N30" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O30" s="45">
+        <v>3.39E-2</v>
+      </c>
+      <c r="P30" s="45">
+        <f t="shared" ref="P30" si="10">O30*M30</f>
+        <v>0.67799999999999994</v>
+      </c>
+      <c r="Q30" s="44"/>
+      <c r="R30" s="49"/>
+    </row>
+    <row r="31" spans="1:18" s="82" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="80"/>
+      <c r="B31" s="39">
+        <f>ROW(B31) - ROW($B$9)</f>
+        <v>22</v>
+      </c>
+      <c r="C31" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="37" t="s">
+        <v>329</v>
+      </c>
+      <c r="G31" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="H31" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="I31" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J31" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="K31" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L31" s="37">
+        <v>1</v>
+      </c>
+      <c r="M31" s="37">
+        <v>2</v>
+      </c>
+      <c r="N31" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O31" s="38">
+        <v>1.4796</v>
+      </c>
+      <c r="P31" s="38">
+        <f>O31*M31</f>
+        <v>2.9592000000000001</v>
+      </c>
+      <c r="Q31" s="37"/>
+      <c r="R31" s="49"/>
+    </row>
+    <row r="32" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="80"/>
+      <c r="B32" s="40">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="C32" s="51"/>
+      <c r="D32" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="F32" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="G32" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="H32" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="I32" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J32" s="44" t="s">
+        <v>343</v>
+      </c>
+      <c r="K32" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L32" s="44">
+        <v>1</v>
+      </c>
+      <c r="M32" s="44">
+        <v>2</v>
+      </c>
+      <c r="N32" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O32" s="45">
+        <v>0.9546</v>
+      </c>
+      <c r="P32" s="45">
+        <f t="shared" ref="P32" si="11">O32*M32</f>
+        <v>1.9092</v>
+      </c>
+      <c r="Q32" s="44"/>
+      <c r="R32" s="49"/>
+    </row>
+    <row r="33" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="80"/>
+      <c r="B33" s="39">
+        <f>ROW(B33) - ROW($B$9)</f>
+        <v>24</v>
+      </c>
+      <c r="C33" s="50" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E33" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="F33" s="37" t="s">
+        <v>329</v>
+      </c>
+      <c r="G33" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="H33" s="37" t="s">
+        <v>228</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J33" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="K33" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L33" s="37">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <v>10</v>
+      </c>
+      <c r="N33" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O33" s="38">
+        <v>4.1300000000000003E-2</v>
+      </c>
+      <c r="P33" s="38">
+        <f>O33*M33</f>
+        <v>0.41300000000000003</v>
+      </c>
+      <c r="Q33" s="37"/>
+      <c r="R33" s="49"/>
+    </row>
+    <row r="34" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="80"/>
+      <c r="B34" s="40">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="C34" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>329</v>
+      </c>
+      <c r="G34" s="44" t="s">
+        <v>150</v>
+      </c>
+      <c r="H34" s="44" t="s">
+        <v>230</v>
+      </c>
+      <c r="I34" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J34" s="44" t="s">
+        <v>269</v>
+      </c>
+      <c r="K34" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L34" s="44">
+        <v>1</v>
+      </c>
+      <c r="M34" s="44">
+        <v>2</v>
+      </c>
+      <c r="N34" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O34" s="45">
+        <v>0.29110000000000003</v>
+      </c>
+      <c r="P34" s="45">
+        <f t="shared" ref="P34" si="12">O34*M34</f>
+        <v>0.58220000000000005</v>
+      </c>
+      <c r="Q34" s="44"/>
+      <c r="R34" s="49"/>
+    </row>
+    <row r="35" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A35" s="80"/>
+      <c r="B35" s="39">
+        <f>ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" s="54" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="F35" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="G35" s="54" t="s">
+        <v>330</v>
+      </c>
+      <c r="H35" s="55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="J35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="K35" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="L35" s="54">
+        <v>13</v>
+      </c>
+      <c r="M35" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="N35" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="O35" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="P35" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q35" s="54"/>
+      <c r="R35" s="58"/>
+    </row>
+    <row r="36" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A36" s="80"/>
+      <c r="B36" s="40">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="C36" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="E36" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="F36" s="44" t="s">
+        <v>151</v>
+      </c>
+      <c r="G36" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="H36" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="I36" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J36" s="44" t="s">
+        <v>270</v>
+      </c>
+      <c r="K36" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L36" s="44">
+        <v>1</v>
+      </c>
+      <c r="M36" s="44">
+        <v>10</v>
+      </c>
+      <c r="N36" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O36" s="45">
+        <v>4.6899999999999997E-2</v>
+      </c>
+      <c r="P36" s="45">
+        <f t="shared" ref="P36" si="13">O36*M36</f>
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="Q36" s="44"/>
+      <c r="R36" s="49"/>
+    </row>
+    <row r="37" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="80"/>
+      <c r="B37" s="39">
+        <f>ROW(B37) - ROW($B$9)</f>
+        <v>28</v>
+      </c>
+      <c r="C37" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="G37" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="H37" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J37" s="37" t="s">
+        <v>271</v>
+      </c>
+      <c r="K37" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="L37" s="37">
+        <v>1</v>
+      </c>
+      <c r="M37" s="37">
+        <v>20</v>
+      </c>
+      <c r="N37" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O37" s="38">
+        <v>3.49E-2</v>
+      </c>
+      <c r="P37" s="38">
+        <f>O37*M37</f>
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="Q37" s="37"/>
+      <c r="R37" s="49"/>
+    </row>
+    <row r="38" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A38" s="80"/>
+      <c r="B38" s="40">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="C38" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="44" t="s">
+        <v>349</v>
+      </c>
+      <c r="E38" s="44" t="s">
+        <v>108</v>
+      </c>
+      <c r="F38" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G38" s="44" t="s">
+        <v>192</v>
+      </c>
+      <c r="H38" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I38" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J38" s="44" t="s">
+        <v>272</v>
+      </c>
+      <c r="K38" s="44" t="s">
+        <v>310</v>
+      </c>
+      <c r="L38" s="44">
+        <v>10</v>
+      </c>
+      <c r="M38" s="44">
+        <v>100</v>
+      </c>
+      <c r="N38" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O38" s="45">
+        <v>1E-3</v>
+      </c>
+      <c r="P38" s="45">
+        <f t="shared" ref="P38" si="14">O38*M38</f>
+        <v>0.1</v>
+      </c>
+      <c r="Q38" s="91" t="s">
+        <v>357</v>
+      </c>
+      <c r="R38" s="49"/>
+    </row>
+    <row r="39" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="80"/>
+      <c r="B39" s="39">
+        <f>ROW(B39) - ROW($B$9)</f>
+        <v>30</v>
+      </c>
+      <c r="C39" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="E39" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="F39" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G39" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="H39" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I39" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J39" s="37" t="s">
+        <v>273</v>
+      </c>
+      <c r="K39" s="37" t="s">
+        <v>311</v>
+      </c>
+      <c r="L39" s="37">
+        <v>3</v>
+      </c>
+      <c r="M39" s="37">
+        <v>100</v>
+      </c>
+      <c r="N39" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O39" s="38">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="P39" s="38">
+        <f>O39*M39</f>
+        <v>0.12</v>
+      </c>
+      <c r="Q39" s="37"/>
+      <c r="R39" s="49"/>
+    </row>
+    <row r="40" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="80"/>
+      <c r="B40" s="40">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="C40" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="44" t="s">
+        <v>110</v>
+      </c>
+      <c r="F40" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G40" s="44" t="s">
+        <v>194</v>
+      </c>
+      <c r="H40" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I40" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J40" s="44" t="s">
+        <v>344</v>
+      </c>
+      <c r="K40" s="44" t="s">
+        <v>312</v>
+      </c>
+      <c r="L40" s="44">
+        <v>3</v>
+      </c>
+      <c r="M40" s="44">
+        <v>100</v>
+      </c>
+      <c r="N40" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O40" s="45">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="P40" s="45">
+        <f t="shared" ref="P40" si="15">O40*M40</f>
+        <v>0.11</v>
+      </c>
+      <c r="Q40" s="44"/>
+      <c r="R40" s="49"/>
+    </row>
+    <row r="41" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="80"/>
+      <c r="B41" s="39">
+        <f>ROW(B41) - ROW($B$9)</f>
+        <v>32</v>
+      </c>
+      <c r="C41" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="F41" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I41" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>274</v>
+      </c>
+      <c r="K41" s="37" t="s">
+        <v>313</v>
+      </c>
+      <c r="L41" s="37">
+        <v>1</v>
+      </c>
+      <c r="M41" s="37">
+        <v>100</v>
+      </c>
+      <c r="N41" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O41" s="38">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="P41" s="38">
+        <f>O41*M41</f>
+        <v>0.12</v>
+      </c>
+      <c r="Q41" s="37"/>
+      <c r="R41" s="49"/>
+    </row>
+    <row r="42" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="80"/>
+      <c r="B42" s="39">
+        <f>ROW(B42) - ROW($B$9)</f>
+        <v>33</v>
+      </c>
+      <c r="C42" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="E42" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="F42" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G42" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="H42" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I42" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J42" s="37" t="s">
+        <v>275</v>
+      </c>
+      <c r="K42" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="L42" s="37">
+        <v>2</v>
+      </c>
+      <c r="M42" s="37">
+        <v>100</v>
+      </c>
+      <c r="N42" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O42" s="38">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="P42" s="38">
+        <f>O42*M42</f>
+        <v>0.11</v>
+      </c>
+      <c r="Q42" s="37"/>
+      <c r="R42" s="49"/>
+    </row>
+    <row r="43" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A43" s="80"/>
+      <c r="B43" s="40">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="C43" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="E43" s="44" t="s">
+        <v>353</v>
+      </c>
+      <c r="F43" s="44" t="s">
+        <v>350</v>
+      </c>
+      <c r="G43" s="44" t="s">
+        <v>351</v>
+      </c>
+      <c r="H43" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I43" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J43" s="44" t="s">
+        <v>352</v>
+      </c>
+      <c r="K43" s="44" t="s">
+        <v>315</v>
+      </c>
+      <c r="L43" s="44">
+        <v>1</v>
+      </c>
+      <c r="M43" s="44">
+        <v>20</v>
+      </c>
+      <c r="N43" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O43" s="45">
+        <v>2.7699999999999999E-2</v>
+      </c>
+      <c r="P43" s="45">
+        <f t="shared" ref="P43" si="16">O43*M43</f>
+        <v>0.55399999999999994</v>
+      </c>
+      <c r="Q43" s="44"/>
+      <c r="R43" s="49"/>
+    </row>
+    <row r="44" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="80"/>
+      <c r="B44" s="39">
+        <f>ROW(B44) - ROW($B$9)</f>
+        <v>35</v>
+      </c>
+      <c r="C44" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D44" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E44" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="F44" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G44" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="H44" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I44" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J44" s="37" t="s">
+        <v>276</v>
+      </c>
+      <c r="K44" s="37" t="s">
+        <v>316</v>
+      </c>
+      <c r="L44" s="37">
+        <v>5</v>
+      </c>
+      <c r="M44" s="37">
+        <v>100</v>
+      </c>
+      <c r="N44" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O44" s="38">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="P44" s="38">
+        <f>O44*M44</f>
+        <v>0.12</v>
+      </c>
+      <c r="Q44" s="37"/>
+      <c r="R44" s="49"/>
+    </row>
+    <row r="45" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="80"/>
+      <c r="B45" s="40">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="C45" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="E45" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="F45" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G45" s="44" t="s">
+        <v>198</v>
+      </c>
+      <c r="H45" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I45" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J45" s="44" t="s">
+        <v>277</v>
+      </c>
+      <c r="K45" s="44" t="s">
+        <v>317</v>
+      </c>
+      <c r="L45" s="44">
+        <v>2</v>
+      </c>
+      <c r="M45" s="44">
+        <v>100</v>
+      </c>
+      <c r="N45" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O45" s="45">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="P45" s="45">
+        <f t="shared" ref="P45" si="17">O45*M45</f>
+        <v>0.31</v>
+      </c>
+      <c r="Q45" s="44"/>
+      <c r="R45" s="49"/>
+    </row>
+    <row r="46" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="80"/>
+      <c r="B46" s="39">
+        <f>ROW(B46) - ROW($B$9)</f>
+        <v>37</v>
+      </c>
+      <c r="C46" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="F46" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G46" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="H46" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I46" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J46" s="37" t="s">
+        <v>278</v>
+      </c>
+      <c r="K46" s="37" t="s">
+        <v>318</v>
+      </c>
+      <c r="L46" s="37">
+        <v>3</v>
+      </c>
+      <c r="M46" s="37">
+        <v>100</v>
+      </c>
+      <c r="N46" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O46" s="38">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="P46" s="38">
+        <f>O46*M46</f>
+        <v>0.11</v>
+      </c>
+      <c r="Q46" s="37"/>
+      <c r="R46" s="49"/>
+    </row>
+    <row r="47" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="80"/>
+      <c r="B47" s="40">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="C47" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="E47" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="F47" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G47" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="H47" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I47" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J47" s="44" t="s">
+        <v>279</v>
+      </c>
+      <c r="K47" s="44" t="s">
+        <v>319</v>
+      </c>
+      <c r="L47" s="44">
+        <v>2</v>
+      </c>
+      <c r="M47" s="44">
+        <v>100</v>
+      </c>
+      <c r="N47" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O47" s="45">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="P47" s="45">
+        <f t="shared" ref="P47" si="18">O47*M47</f>
+        <v>0.12</v>
+      </c>
+      <c r="Q47" s="44"/>
+      <c r="R47" s="49"/>
+    </row>
+    <row r="48" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="80"/>
+      <c r="B48" s="39">
+        <f>ROW(B48) - ROW($B$9)</f>
+        <v>39</v>
+      </c>
+      <c r="C48" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D48" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="F48" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G48" s="37" t="s">
+        <v>201</v>
+      </c>
+      <c r="H48" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I48" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J48" s="37" t="s">
+        <v>280</v>
+      </c>
+      <c r="K48" s="37" t="s">
+        <v>320</v>
+      </c>
+      <c r="L48" s="37">
+        <v>2</v>
+      </c>
+      <c r="M48" s="37">
+        <v>100</v>
+      </c>
+      <c r="N48" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O48" s="38">
+        <v>1.8E-3</v>
+      </c>
+      <c r="P48" s="38">
+        <f>O48*M48</f>
+        <v>0.18</v>
+      </c>
+      <c r="Q48" s="37"/>
+      <c r="R48" s="49"/>
+    </row>
+    <row r="49" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A49" s="80"/>
+      <c r="B49" s="40">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="C49" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="E49" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="F49" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G49" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="H49" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I49" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J49" s="44" t="s">
+        <v>281</v>
+      </c>
+      <c r="K49" s="44" t="s">
+        <v>321</v>
+      </c>
+      <c r="L49" s="44">
+        <v>1</v>
+      </c>
+      <c r="M49" s="44">
+        <v>20</v>
+      </c>
+      <c r="N49" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O49" s="45">
+        <v>2.75E-2</v>
+      </c>
+      <c r="P49" s="45">
+        <f t="shared" ref="P49" si="19">O49*M49</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="Q49" s="44"/>
+      <c r="R49" s="49"/>
+    </row>
+    <row r="50" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="80"/>
+      <c r="B50" s="39">
+        <f>ROW(B50) - ROW($B$9)</f>
+        <v>41</v>
+      </c>
+      <c r="C50" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="E50" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="F50" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G50" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="H50" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I50" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J50" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="K50" s="37" t="s">
+        <v>322</v>
+      </c>
+      <c r="L50" s="37">
+        <v>1</v>
+      </c>
+      <c r="M50" s="37">
+        <v>50</v>
+      </c>
+      <c r="N50" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O50" s="38">
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="P50" s="38">
+        <f>O50*M50</f>
+        <v>0.44</v>
+      </c>
+      <c r="Q50" s="37"/>
+      <c r="R50" s="49"/>
+    </row>
+    <row r="51" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="80"/>
+      <c r="B51" s="40">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C51" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="44" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="F51" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G51" s="44" t="s">
+        <v>204</v>
+      </c>
+      <c r="H51" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I51" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J51" s="44" t="s">
+        <v>283</v>
+      </c>
+      <c r="K51" s="44" t="s">
+        <v>323</v>
+      </c>
+      <c r="L51" s="44">
+        <v>1</v>
+      </c>
+      <c r="M51" s="44">
+        <v>20</v>
+      </c>
+      <c r="N51" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O51" s="45">
+        <v>2.63E-2</v>
+      </c>
+      <c r="P51" s="45">
+        <f t="shared" ref="P51" si="20">O51*M51</f>
+        <v>0.52600000000000002</v>
+      </c>
+      <c r="Q51" s="44"/>
+      <c r="R51" s="49"/>
+    </row>
+    <row r="52" spans="1:18" s="90" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="83"/>
+      <c r="B52" s="84">
+        <f>ROW(B52) - ROW($B$9)</f>
+        <v>43</v>
+      </c>
+      <c r="C52" s="85" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="86" t="s">
+        <v>64</v>
+      </c>
+      <c r="E52" s="86" t="s">
+        <v>121</v>
+      </c>
+      <c r="F52" s="86" t="s">
+        <v>152</v>
+      </c>
+      <c r="G52" s="86" t="s">
+        <v>205</v>
+      </c>
+      <c r="H52" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="I52" s="86" t="s">
+        <v>328</v>
+      </c>
+      <c r="J52" s="86" t="s">
+        <v>284</v>
+      </c>
+      <c r="K52" s="86" t="s">
+        <v>324</v>
+      </c>
+      <c r="L52" s="86">
+        <v>1</v>
+      </c>
+      <c r="M52" s="86">
+        <v>20</v>
+      </c>
+      <c r="N52" s="87" t="s">
+        <v>342</v>
+      </c>
+      <c r="O52" s="88">
+        <v>3.1E-2</v>
+      </c>
+      <c r="P52" s="88">
+        <f>O52*M52</f>
+        <v>0.62</v>
+      </c>
+      <c r="Q52" s="86"/>
+      <c r="R52" s="89"/>
+    </row>
+    <row r="53" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="80"/>
+      <c r="B53" s="40">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C53" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="E53" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="F53" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="G53" s="44" t="s">
+        <v>206</v>
+      </c>
+      <c r="H53" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="I53" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J53" s="44" t="s">
+        <v>285</v>
+      </c>
+      <c r="K53" s="44" t="s">
+        <v>325</v>
+      </c>
+      <c r="L53" s="44">
+        <v>1</v>
+      </c>
+      <c r="M53" s="44">
+        <v>100</v>
+      </c>
+      <c r="N53" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O53" s="45">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="P53" s="45">
+        <f t="shared" ref="P53" si="21">O53*M53</f>
+        <v>0.12</v>
+      </c>
+      <c r="Q53" s="44"/>
+      <c r="R53" s="49"/>
+    </row>
+    <row r="54" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="80"/>
+      <c r="B54" s="39">
+        <f>ROW(B54) - ROW($B$9)</f>
+        <v>45</v>
+      </c>
+      <c r="C54" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="D54" s="54" t="s">
+        <v>66</v>
+      </c>
+      <c r="E54" s="54" t="s">
+        <v>123</v>
+      </c>
+      <c r="F54" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="G54" s="54" t="s">
+        <v>153</v>
+      </c>
+      <c r="H54" s="55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="J54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="K54" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="L54" s="54">
+        <v>3</v>
+      </c>
+      <c r="M54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="N54" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="O54" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="P54" s="57" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q54" s="54"/>
+      <c r="R54" s="58"/>
+    </row>
+    <row r="55" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="80"/>
+      <c r="B55" s="40">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="C55" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="E55" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="F55" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="G55" s="44" t="s">
+        <v>154</v>
+      </c>
+      <c r="H55" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="I55" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J55" s="44" t="s">
+        <v>286</v>
+      </c>
+      <c r="K55" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L55" s="44">
+        <v>5</v>
+      </c>
+      <c r="M55" s="44">
+        <v>10</v>
+      </c>
+      <c r="N55" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O55" s="45">
+        <v>0.3135</v>
+      </c>
+      <c r="P55" s="45">
+        <f t="shared" ref="P55:P56" si="22">O55*M55</f>
+        <v>3.1349999999999998</v>
+      </c>
+      <c r="Q55" s="44"/>
+      <c r="R55" s="49"/>
+    </row>
+    <row r="56" spans="1:18" s="82" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A56" s="80"/>
+      <c r="B56" s="40">
+        <f>ROW(B56) - ROW($B$9)</f>
+        <v>47</v>
+      </c>
+      <c r="C56" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="44" t="s">
+        <v>327</v>
+      </c>
+      <c r="E56" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F56" s="44" t="s">
+        <v>329</v>
+      </c>
+      <c r="G56" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="H56" s="44" t="s">
+        <v>240</v>
+      </c>
+      <c r="I56" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J56" s="44" t="s">
+        <v>291</v>
+      </c>
+      <c r="K56" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L56" s="44">
+        <v>1</v>
+      </c>
+      <c r="M56" s="44">
+        <v>10</v>
+      </c>
+      <c r="N56" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O56" s="45">
+        <v>6.2100000000000002E-2</v>
+      </c>
+      <c r="P56" s="45">
+        <f t="shared" si="22"/>
+        <v>0.621</v>
+      </c>
+      <c r="Q56" s="44"/>
+      <c r="R56" s="49"/>
+    </row>
+    <row r="57" spans="1:18" s="82" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A57" s="80"/>
+      <c r="B57" s="39">
+        <f>ROW(B57) - ROW($B$9)</f>
+        <v>48</v>
+      </c>
+      <c r="C57" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="E57" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="F57" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="G57" s="37" t="s">
+        <v>207</v>
+      </c>
+      <c r="H57" s="37" t="s">
+        <v>235</v>
+      </c>
+      <c r="I57" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J57" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="K57" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L57" s="37">
+        <v>1</v>
+      </c>
+      <c r="M57" s="37">
+        <v>2</v>
+      </c>
+      <c r="N57" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O57" s="38">
+        <v>0.16209999999999999</v>
+      </c>
+      <c r="P57" s="38">
+        <f>O57*M57</f>
+        <v>0.32419999999999999</v>
+      </c>
+      <c r="Q57" s="37"/>
+      <c r="R57" s="49"/>
+    </row>
+    <row r="58" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="80"/>
+      <c r="B58" s="40">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="C58" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="F58" s="44" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="H58" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="I58" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J58" s="44" t="s">
+        <v>348</v>
+      </c>
+      <c r="K58" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L58" s="44">
+        <v>1</v>
+      </c>
+      <c r="M58" s="44">
+        <v>5</v>
+      </c>
+      <c r="N58" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O58" s="45">
+        <v>0.1341</v>
+      </c>
+      <c r="P58" s="45">
+        <f t="shared" ref="P58" si="23">O58*M58</f>
+        <v>0.67049999999999998</v>
+      </c>
+      <c r="Q58" s="44"/>
+      <c r="R58" s="49"/>
+    </row>
+    <row r="59" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A59" s="80"/>
+      <c r="B59" s="39">
+        <f>ROW(B59) - ROW($B$9)</f>
+        <v>50</v>
+      </c>
+      <c r="C59" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="E59" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="F59" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="G59" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="H59" s="37" t="s">
+        <v>237</v>
+      </c>
+      <c r="I59" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J59" s="37" t="s">
+        <v>288</v>
+      </c>
+      <c r="K59" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L59" s="37">
+        <v>1</v>
+      </c>
+      <c r="M59" s="37">
+        <v>5</v>
+      </c>
+      <c r="N59" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O59" s="38">
+        <v>0.19539999999999999</v>
+      </c>
+      <c r="P59" s="38">
+        <f>O59*M59</f>
+        <v>0.97699999999999998</v>
+      </c>
+      <c r="Q59" s="37"/>
+      <c r="R59" s="49"/>
+    </row>
+    <row r="60" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A60" s="80"/>
+      <c r="B60" s="40">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="C60" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="E60" s="44" t="s">
+        <v>128</v>
+      </c>
+      <c r="F60" s="44" t="s">
+        <v>158</v>
+      </c>
+      <c r="G60" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="H60" s="44" t="s">
+        <v>238</v>
+      </c>
+      <c r="I60" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J60" s="44" t="s">
+        <v>289</v>
+      </c>
+      <c r="K60" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L60" s="44">
+        <v>1</v>
+      </c>
+      <c r="M60" s="44">
+        <v>2</v>
+      </c>
+      <c r="N60" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O60" s="45">
+        <v>0.43909999999999999</v>
+      </c>
+      <c r="P60" s="45">
+        <f t="shared" ref="P60" si="24">O60*M60</f>
+        <v>0.87819999999999998</v>
+      </c>
+      <c r="Q60" s="44"/>
+      <c r="R60" s="49"/>
+    </row>
+    <row r="61" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A61" s="80"/>
+      <c r="B61" s="39">
+        <f>ROW(B61) - ROW($B$9)</f>
+        <v>52</v>
+      </c>
+      <c r="C61" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D61" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="E61" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="F61" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="G61" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="H61" s="37" t="s">
+        <v>239</v>
+      </c>
+      <c r="I61" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J61" s="37" t="s">
+        <v>290</v>
+      </c>
+      <c r="K61" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L61" s="37">
+        <v>1</v>
+      </c>
+      <c r="M61" s="37">
+        <v>5</v>
+      </c>
+      <c r="N61" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O61" s="38">
+        <v>0.15479999999999999</v>
+      </c>
+      <c r="P61" s="38">
+        <f>O61*M61</f>
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="Q61" s="37"/>
+      <c r="R61" s="49"/>
+    </row>
+    <row r="62" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A62" s="80"/>
+      <c r="B62" s="39">
+        <f>ROW(B62) - ROW($B$9)</f>
+        <v>53</v>
+      </c>
+      <c r="C62" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="D62" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="E62" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="F62" s="37" t="s">
+        <v>161</v>
+      </c>
+      <c r="G62" s="37" t="s">
+        <v>212</v>
+      </c>
+      <c r="H62" s="37" t="s">
+        <v>241</v>
+      </c>
+      <c r="I62" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J62" s="37" t="s">
+        <v>292</v>
+      </c>
+      <c r="K62" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L62" s="37">
+        <v>1</v>
+      </c>
+      <c r="M62" s="37">
+        <v>2</v>
+      </c>
+      <c r="N62" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O62" s="38">
+        <v>5.1212</v>
+      </c>
+      <c r="P62" s="38">
+        <f>O62*M62</f>
+        <v>10.2424</v>
+      </c>
+      <c r="Q62" s="37"/>
+      <c r="R62" s="49"/>
+    </row>
+    <row r="63" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A63" s="80"/>
+      <c r="B63" s="40">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="C63" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D63" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="E63" s="44" t="s">
+        <v>132</v>
+      </c>
+      <c r="F63" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="G63" s="44" t="s">
+        <v>213</v>
+      </c>
+      <c r="H63" s="44" t="s">
+        <v>242</v>
+      </c>
+      <c r="I63" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J63" s="44" t="s">
+        <v>293</v>
+      </c>
+      <c r="K63" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L63" s="44">
+        <v>1</v>
+      </c>
+      <c r="M63" s="44">
+        <v>5</v>
+      </c>
+      <c r="N63" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O63" s="45">
+        <v>0.15670000000000001</v>
+      </c>
+      <c r="P63" s="45">
+        <f t="shared" ref="P63" si="25">O63*M63</f>
+        <v>0.78350000000000009</v>
+      </c>
+      <c r="Q63" s="44"/>
+      <c r="R63" s="49"/>
+    </row>
+    <row r="64" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A64" s="80"/>
+      <c r="B64" s="39">
+        <f>ROW(B64) - ROW($B$9)</f>
+        <v>55</v>
+      </c>
+      <c r="C64" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="E64" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="F64" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="G64" s="37" t="s">
+        <v>214</v>
+      </c>
+      <c r="H64" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="I64" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J64" s="37" t="s">
+        <v>294</v>
+      </c>
+      <c r="K64" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L64" s="37">
+        <v>1</v>
+      </c>
+      <c r="M64" s="37">
+        <v>2</v>
+      </c>
+      <c r="N64" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O64" s="38">
+        <v>0.96889999999999998</v>
+      </c>
+      <c r="P64" s="38">
+        <f>O64*M64</f>
+        <v>1.9378</v>
+      </c>
+      <c r="Q64" s="37"/>
+      <c r="R64" s="49"/>
+    </row>
+    <row r="65" spans="1:18" s="82" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="80"/>
+      <c r="B65" s="40">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="C65" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D65" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="E65" s="44" t="s">
+        <v>134</v>
+      </c>
+      <c r="F65" s="44" t="s">
+        <v>164</v>
+      </c>
+      <c r="G65" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="H65" s="44" t="s">
+        <v>244</v>
+      </c>
+      <c r="I65" s="44" t="s">
+        <v>328</v>
+      </c>
+      <c r="J65" s="44" t="s">
+        <v>295</v>
+      </c>
+      <c r="K65" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L65" s="44">
+        <v>1</v>
+      </c>
+      <c r="M65" s="44">
+        <v>2</v>
+      </c>
+      <c r="N65" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="O65" s="45">
+        <v>0.28870000000000001</v>
+      </c>
+      <c r="P65" s="45">
+        <f t="shared" ref="P65" si="26">O65*M65</f>
+        <v>0.57740000000000002</v>
+      </c>
+      <c r="Q65" s="44"/>
+      <c r="R65" s="49"/>
+    </row>
+    <row r="66" spans="1:18" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A66" s="80"/>
+      <c r="B66" s="39">
+        <f>ROW(B66) - ROW($B$9)</f>
+        <v>57</v>
+      </c>
+      <c r="C66" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D66" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E66" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="F66" s="37" t="s">
+        <v>165</v>
+      </c>
+      <c r="G66" s="37" t="s">
+        <v>216</v>
+      </c>
+      <c r="H66" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="I66" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="J66" s="37" t="s">
+        <v>296</v>
+      </c>
+      <c r="K66" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="L66" s="37">
+        <v>1</v>
+      </c>
+      <c r="M66" s="37">
+        <v>2</v>
+      </c>
+      <c r="N66" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="O66" s="38">
+        <v>2.0651000000000002</v>
+      </c>
+      <c r="P66" s="38">
+        <f>O66*M66</f>
+        <v>4.1302000000000003</v>
+      </c>
+      <c r="Q66" s="37"/>
+      <c r="R66" s="49"/>
+    </row>
+    <row r="67" spans="1:18" s="82" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="80"/>
+      <c r="B67" s="59">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="C67" s="60" t="s">
+        <v>21</v>
+      </c>
+      <c r="D67" s="49" t="s">
+        <v>78</v>
+      </c>
+      <c r="E67" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="F67" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="G67" s="49" t="s">
+        <v>217</v>
+      </c>
+      <c r="H67" s="49" t="s">
+        <v>245</v>
+      </c>
+      <c r="I67" s="49" t="s">
+        <v>328</v>
+      </c>
+      <c r="J67" s="49" t="s">
+        <v>297</v>
+      </c>
+      <c r="K67" s="61" t="s">
+        <v>328</v>
+      </c>
+      <c r="L67" s="49">
+        <v>1</v>
+      </c>
+      <c r="M67" s="49">
+        <v>2</v>
+      </c>
+      <c r="N67" s="62" t="s">
+        <v>342</v>
+      </c>
+      <c r="O67" s="63">
+        <v>1.2919</v>
+      </c>
+      <c r="P67" s="63">
+        <f t="shared" ref="P67" si="27">O67*M67</f>
+        <v>2.5838000000000001</v>
+      </c>
+      <c r="Q67" s="49"/>
+      <c r="R67" s="49"/>
+    </row>
+    <row r="68" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="1"/>
+      <c r="B68" s="93"/>
+      <c r="C68" s="94"/>
+      <c r="D68" s="95"/>
+      <c r="E68" s="96"/>
+      <c r="F68" s="97"/>
+      <c r="G68" s="98"/>
+      <c r="H68" s="97"/>
+      <c r="I68" s="98"/>
+      <c r="J68" s="97"/>
+      <c r="K68" s="98"/>
+      <c r="L68" s="98"/>
+      <c r="M68" s="78" t="s">
+        <v>5</v>
+      </c>
+      <c r="N68" s="79"/>
+      <c r="O68" s="79"/>
+      <c r="P68" s="41">
+        <f>SUM(P10:P67)</f>
+        <v>55.211800000000011</v>
+      </c>
+      <c r="Q68" s="99"/>
+      <c r="R68" s="100"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="K1:R1"/>
+    <mergeCell ref="R3:R8"/>
+    <mergeCell ref="M68:O68"/>
+    <mergeCell ref="Q68:R68"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="N10" r:id="rId1"/>
+    <hyperlink ref="N11" r:id="rId2"/>
+    <hyperlink ref="N12" r:id="rId3"/>
+    <hyperlink ref="N13" r:id="rId4"/>
+    <hyperlink ref="N14" r:id="rId5"/>
+    <hyperlink ref="N15" r:id="rId6"/>
+    <hyperlink ref="N16" r:id="rId7"/>
+    <hyperlink ref="N17" r:id="rId8"/>
+    <hyperlink ref="N19" r:id="rId9"/>
+    <hyperlink ref="N20" r:id="rId10"/>
+    <hyperlink ref="N21" r:id="rId11"/>
+    <hyperlink ref="N22" r:id="rId12"/>
+    <hyperlink ref="N23" r:id="rId13"/>
+    <hyperlink ref="N24" r:id="rId14"/>
+    <hyperlink ref="N25" r:id="rId15"/>
+    <hyperlink ref="N26" r:id="rId16"/>
+    <hyperlink ref="N27" r:id="rId17"/>
+    <hyperlink ref="N28" r:id="rId18"/>
+    <hyperlink ref="N29" r:id="rId19"/>
+    <hyperlink ref="N30" r:id="rId20"/>
+    <hyperlink ref="N31" r:id="rId21"/>
+    <hyperlink ref="N32" r:id="rId22"/>
+    <hyperlink ref="N33" r:id="rId23"/>
+    <hyperlink ref="N34" r:id="rId24"/>
+    <hyperlink ref="N36" r:id="rId25"/>
+    <hyperlink ref="N37" r:id="rId26"/>
+    <hyperlink ref="N38" r:id="rId27"/>
+    <hyperlink ref="N39" r:id="rId28"/>
+    <hyperlink ref="N40" r:id="rId29"/>
+    <hyperlink ref="N41" r:id="rId30"/>
+    <hyperlink ref="N42" r:id="rId31"/>
+    <hyperlink ref="N44" r:id="rId32"/>
+    <hyperlink ref="N45" r:id="rId33"/>
+    <hyperlink ref="N46" r:id="rId34"/>
+    <hyperlink ref="N47" r:id="rId35"/>
+    <hyperlink ref="N48" r:id="rId36"/>
+    <hyperlink ref="N49" r:id="rId37"/>
+    <hyperlink ref="N50" r:id="rId38"/>
+    <hyperlink ref="N51" r:id="rId39"/>
+    <hyperlink ref="N52" r:id="rId40"/>
+    <hyperlink ref="N53" r:id="rId41"/>
+    <hyperlink ref="N55" r:id="rId42"/>
+    <hyperlink ref="N56" r:id="rId43"/>
+    <hyperlink ref="N57" r:id="rId44"/>
+    <hyperlink ref="N59" r:id="rId45"/>
+    <hyperlink ref="N60" r:id="rId46"/>
+    <hyperlink ref="N61" r:id="rId47"/>
+    <hyperlink ref="N62" r:id="rId48"/>
+    <hyperlink ref="N63" r:id="rId49"/>
+    <hyperlink ref="N64" r:id="rId50"/>
+    <hyperlink ref="N65" r:id="rId51"/>
+    <hyperlink ref="N66" r:id="rId52"/>
+    <hyperlink ref="N67" r:id="rId53"/>
+    <hyperlink ref="N18" r:id="rId54"/>
+    <hyperlink ref="N58" r:id="rId55"/>
+    <hyperlink ref="N43" r:id="rId56"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId57"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S69"/>
+  <dimension ref="A1:S70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -3995,7 +7492,9 @@
         <f t="shared" ref="Q38" si="30">P38*N38</f>
         <v>0.1</v>
       </c>
-      <c r="R38" s="44"/>
+      <c r="R38" s="91" t="s">
+        <v>357</v>
+      </c>
       <c r="S38" s="49"/>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
@@ -5672,6 +9171,9 @@
       </c>
       <c r="R69" s="76"/>
       <c r="S69" s="77"/>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="P70" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>